<commit_message>
Update DATA_COST_FOB from Cost Fob.xlsx - new values from Quy cách khác sheet
</commit_message>
<xml_diff>
--- a/sites/kiem-tra-gia/data/Cost Fob.xlsx
+++ b/sites/kiem-tra-gia/data/Cost Fob.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\.openclaw\workspace-skills\web-builder\sites\kiem-tra-gia\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C91B4BE2-98C3-4710-9750-3615A2337FE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{100EC5A2-915B-46D0-843D-A4E43175BE8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="26537" windowHeight="14297" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -450,10 +450,10 @@
         <v>14</v>
       </c>
       <c r="B2" s="3">
-        <v>1005400</v>
+        <v>974600</v>
       </c>
       <c r="C2" s="3">
-        <v>1294700</v>
+        <v>1263900</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="15.45" x14ac:dyDescent="0.4">
@@ -461,10 +461,10 @@
         <v>20</v>
       </c>
       <c r="B3" s="3">
-        <v>704840</v>
+        <v>682000</v>
       </c>
       <c r="C3" s="3">
-        <v>907350</v>
+        <v>884400</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="15.45" x14ac:dyDescent="0.4">
@@ -472,10 +472,10 @@
         <v>22</v>
       </c>
       <c r="B4" s="3">
-        <v>640200</v>
+        <v>620400</v>
       </c>
       <c r="C4" s="3">
-        <v>823900</v>
+        <v>804100</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="15.45" x14ac:dyDescent="0.4">
@@ -483,10 +483,10 @@
         <v>24</v>
       </c>
       <c r="B5" s="3">
-        <v>586300</v>
+        <v>568700</v>
       </c>
       <c r="C5" s="3">
-        <v>755700</v>
+        <v>737000</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="15.45" x14ac:dyDescent="0.4">
@@ -494,10 +494,10 @@
         <v>25</v>
       </c>
       <c r="B6" s="3">
-        <v>563200</v>
+        <v>545600</v>
       </c>
       <c r="C6" s="3">
-        <v>726000</v>
+        <v>707300</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="15.45" x14ac:dyDescent="0.4">
@@ -505,10 +505,10 @@
         <v>26</v>
       </c>
       <c r="B7" s="3">
-        <v>541200</v>
+        <v>524700</v>
       </c>
       <c r="C7" s="3">
-        <v>697400</v>
+        <v>680900</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="15.45" x14ac:dyDescent="0.4">
@@ -516,10 +516,10 @@
         <v>27</v>
       </c>
       <c r="B8" s="3">
-        <v>521400</v>
+        <v>504900</v>
       </c>
       <c r="C8" s="3">
-        <v>672100</v>
+        <v>655600</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="15.45" x14ac:dyDescent="0.4">
@@ -527,13 +527,14 @@
         <v>28</v>
       </c>
       <c r="B9" s="3">
-        <v>502700</v>
+        <v>487300</v>
       </c>
       <c r="C9" s="3">
-        <v>647900</v>
+        <v>632500</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: CostFOB import Vietnamese columns, rename sheet to CostFOB
</commit_message>
<xml_diff>
--- a/sites/kiem-tra-gia/data/Cost Fob.xlsx
+++ b/sites/kiem-tra-gia/data/Cost Fob.xlsx
@@ -1,80 +1,48 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\.openclaw\workspace-skills\web-builder\sites\kiem-tra-gia\data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{100EC5A2-915B-46D0-843D-A4E43175BE8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="26537" windowHeight="14297" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-103" yWindow="-103" windowWidth="26537" windowHeight="14297" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Quy cách khác" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CostFOB" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
-  <si>
-    <t>Max loadding</t>
-  </si>
-  <si>
-    <t>No LCC</t>
-  </si>
-  <si>
-    <t>Sub LCC</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="12"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Cambria"/>
       <family val="1"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="12"/>
       <scheme val="major"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Cambria"/>
       <family val="1"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="major"/>
     </font>
   </fonts>
   <fills count="3">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -114,30 +82,89 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -425,116 +452,126 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.6"/>
   <cols>
-    <col min="1" max="1" width="22.3828125" customWidth="1"/>
-    <col min="2" max="2" width="17" customWidth="1"/>
-    <col min="3" max="3" width="11.3828125" customWidth="1"/>
+    <col width="22.3828125" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="11.3828125" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15" x14ac:dyDescent="0.4">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="15.45" x14ac:dyDescent="0.4">
-      <c r="A2" s="2">
+    <row r="1" ht="15" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Max loadding</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>No LCC</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Sub LCC</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15.45" customHeight="1">
+      <c r="A2" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="3" t="n">
         <v>974600</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="3" t="n">
         <v>1263900</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="15.45" x14ac:dyDescent="0.4">
-      <c r="A3" s="2">
+    <row r="3" ht="15.45" customHeight="1">
+      <c r="A3" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="3" t="n">
         <v>682000</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="3" t="n">
         <v>884400</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15.45" x14ac:dyDescent="0.4">
-      <c r="A4" s="2">
+    <row r="4" ht="15.45" customHeight="1">
+      <c r="A4" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="3" t="n">
         <v>620400</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="3" t="n">
         <v>804100</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="15.45" x14ac:dyDescent="0.4">
-      <c r="A5" s="2">
+    <row r="5" ht="15.45" customHeight="1">
+      <c r="A5" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="3" t="n">
         <v>568700</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="3" t="n">
         <v>737000</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15.45" x14ac:dyDescent="0.4">
-      <c r="A6" s="2">
+    <row r="6" ht="15.45" customHeight="1">
+      <c r="A6" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="3" t="n">
         <v>545600</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="3" t="n">
         <v>707300</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="15.45" x14ac:dyDescent="0.4">
-      <c r="A7" s="2">
+    <row r="7" ht="15.45" customHeight="1">
+      <c r="A7" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7" s="3" t="n">
         <v>524700</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="3" t="n">
         <v>680900</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="15.45" x14ac:dyDescent="0.4">
-      <c r="A8" s="2">
+    <row r="8" ht="15.45" customHeight="1">
+      <c r="A8" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B8" s="3" t="n">
         <v>504900</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="3" t="n">
         <v>655600</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="15.45" x14ac:dyDescent="0.4">
-      <c r="A9" s="2">
+    <row r="9" ht="15.45" customHeight="1">
+      <c r="A9" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="B9" s="3">
+      <c r="B9" s="3" t="n">
         <v>487300</v>
       </c>
-      <c r="C9" s="3">
+      <c r="C9" s="3" t="n">
         <v>632500</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: rebuild Cost Fob.xlsx with XLSX for correct header/Latin chars
</commit_message>
<xml_diff>
--- a/sites/kiem-tra-gia/data/Cost Fob.xlsx
+++ b/sites/kiem-tra-gia/data/Cost Fob.xlsx
@@ -1,60 +1,58 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-103" yWindow="-103" windowWidth="26537" windowHeight="14297" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CostFOB" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="CostFOB" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <numFmts count="1">
+    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+  </numFmts>
+  <fonts count="1">
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <name val="Cambria"/>
-      <family val="1"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="12"/>
-      <scheme val="major"/>
-    </font>
-    <font>
-      <name val="Cambria"/>
-      <family val="1"/>
-      <color theme="1"/>
-      <sz val="12"/>
-      <scheme val="major"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1A56DB"/>
-        <bgColor rgb="FF1A56DB"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -62,109 +60,18 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
 </styleSheet>
 </file>
 
@@ -243,6 +150,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -277,6 +185,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -311,20 +220,16 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -446,132 +351,156 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.6"/>
-  <cols>
-    <col width="22.3828125" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="11.3828125" customWidth="1" min="3" max="3"/>
-  </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Max loadding</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>No LCC</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Sub LCC</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="15.45" customHeight="1">
-      <c r="A2" s="2" t="n">
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Max loadding</v>
+      </c>
+      <c r="B1" t="str">
+        <v>No LCC</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Sub LCC</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
         <v>14</v>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B2">
         <v>974600</v>
       </c>
-      <c r="C2" s="3" t="n">
+      <c r="C2">
         <v>1263900</v>
       </c>
     </row>
-    <row r="3" ht="15.45" customHeight="1">
-      <c r="A3" s="2" t="n">
+    <row r="3">
+      <c r="A3">
         <v>20</v>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B3">
         <v>682000</v>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="C3">
         <v>884400</v>
       </c>
     </row>
-    <row r="4" ht="15.45" customHeight="1">
-      <c r="A4" s="2" t="n">
+    <row r="4">
+      <c r="A4">
         <v>22</v>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B4">
         <v>620400</v>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="C4">
         <v>804100</v>
       </c>
     </row>
-    <row r="5" ht="15.45" customHeight="1">
-      <c r="A5" s="2" t="n">
+    <row r="5">
+      <c r="A5">
         <v>24</v>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B5">
         <v>568700</v>
       </c>
-      <c r="C5" s="3" t="n">
+      <c r="C5">
         <v>737000</v>
       </c>
     </row>
-    <row r="6" ht="15.45" customHeight="1">
-      <c r="A6" s="2" t="n">
+    <row r="6">
+      <c r="A6">
         <v>25</v>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B6">
         <v>545600</v>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="C6">
         <v>707300</v>
       </c>
     </row>
-    <row r="7" ht="15.45" customHeight="1">
-      <c r="A7" s="2" t="n">
+    <row r="7">
+      <c r="A7">
         <v>26</v>
       </c>
-      <c r="B7" s="3" t="n">
+      <c r="B7">
         <v>524700</v>
       </c>
-      <c r="C7" s="3" t="n">
+      <c r="C7">
         <v>680900</v>
       </c>
     </row>
-    <row r="8" ht="15.45" customHeight="1">
-      <c r="A8" s="2" t="n">
+    <row r="8">
+      <c r="A8">
         <v>27</v>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B8">
         <v>504900</v>
       </c>
-      <c r="C8" s="3" t="n">
+      <c r="C8">
         <v>655600</v>
       </c>
     </row>
-    <row r="9" ht="15.45" customHeight="1">
-      <c r="A9" s="2" t="n">
+    <row r="9">
+      <c r="A9">
         <v>28</v>
       </c>
-      <c r="B9" s="3" t="n">
+      <c r="B9">
         <v>487300</v>
       </c>
-      <c r="C9" s="3" t="n">
+      <c r="C9">
         <v>632500</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C9"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: remove orphan subrows on filter change, preview popup uses self-contained generator
</commit_message>
<xml_diff>
--- a/sites/kiem-tra-gia/data/Cost Fob.xlsx
+++ b/sites/kiem-tra-gia/data/Cost Fob.xlsx
@@ -1,41 +1,54 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\.openclaw\workspace-skills\web-builder\sites\kiem-tra-gia\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_C5F30130CC387D6A206102340812B83BA12CD052" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="26537" windowHeight="14297" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="CostFOB" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+  <si>
+    <t>Max loadding</t>
+  </si>
+  <si>
+    <t>No LCC</t>
+  </si>
+  <si>
+    <t>Sub LCC</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -65,13 +78,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,21 +417,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Max loadding</v>
-      </c>
-      <c r="B1" t="str">
-        <v>No LCC</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Sub LCC</v>
-      </c>
-    </row>
-    <row r="2">
+    <row r="1" spans="1:3" ht="15.9" x14ac:dyDescent="0.45">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="15.9" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>14</v>
       </c>
@@ -421,7 +443,7 @@
         <v>1263900</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:3" ht="15.9" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>20</v>
       </c>
@@ -432,7 +454,7 @@
         <v>884400</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:3" ht="15.9" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>22</v>
       </c>
@@ -443,7 +465,7 @@
         <v>804100</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:3" ht="15.9" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>24</v>
       </c>
@@ -454,7 +476,7 @@
         <v>737000</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:3" ht="15.9" x14ac:dyDescent="0.45">
       <c r="A6">
         <v>25</v>
       </c>
@@ -465,7 +487,7 @@
         <v>707300</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:3" ht="15.9" x14ac:dyDescent="0.45">
       <c r="A7">
         <v>26</v>
       </c>
@@ -476,7 +498,7 @@
         <v>680900</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:3" ht="15.9" x14ac:dyDescent="0.45">
       <c r="A8">
         <v>27</v>
       </c>
@@ -487,7 +509,7 @@
         <v>655600</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:3" ht="15.9" x14ac:dyDescent="0.45">
       <c r="A9">
         <v>28</v>
       </c>
@@ -499,8 +521,9 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C9"/>
+    <ignoredError sqref="A1:C9" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>